<commit_message>
Add Barton elastoplastic solid validation solver
Added an elastoplastic solid modelling module based on the Barton formulation.

Implemented a unified solid_main entry point and a Barton solver structure split by responsibility: state, EOS, flux, plasticity, advance, config, output, initial conditions, and driver. Added 1D flyer-plate validation cases and a 2D radial-pressure tensor validation case, with plotting scripts for the Barton stress/time figures and Figure 6-style radial comparisons.

Cleaned the solid folder structure so validation configs are separated from solver code, removed legacy solid paths, and documented the current solid layout in docs/solid_refactor_report.md.

Validation run:
- Barton 1D test1: 609 steps, final_time = 5e-06
- Barton 1D test2: 731 steps, final_time = 5e-06
- Barton 2D debug: 86 steps, final_time = 1e-05
- Solid plots regenerated successfully
- Existing Toro 1D Euler path still compiles and runs
</commit_message>
<xml_diff>
--- a/data/bubble_collapse_validation/2d bubble collapse.xlsx
+++ b/data/bubble_collapse_validation/2d bubble collapse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\oluse\diffuse_vs_GFM_MMS\data\bubble_collapse_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86F0C3E-1984-4B2B-965E-F43E66F120D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A330E16-10C1-4F05-A963-D010DB009C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" activeTab="1" xr2:uid="{EDC50580-E04D-44B0-82D6-6934DBA8A6C2}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{EDC50580-E04D-44B0-82D6-6934DBA8A6C2}"/>
   </bookViews>
   <sheets>
     <sheet name="GFM" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Move bubble feature tracking into src and wire quantitative runner
Moved the helium shock-bubble feature tracking tools from analysis into src/bubble_features, added explanatory comments for the feature definitions and temporal branch tracking, and wired the workflow into scripts/run_quant_suite.sh.

The runner now supports optional bubble feature extraction via --bubble-features or --bubble-only, including GFM/SIM and DIM/Allaire outputs. The batch pipeline writes master feature positions, transmitted shock/upstream candidate diagnostics, selected temporal branches, overlays, and velocity fits.
</commit_message>
<xml_diff>
--- a/data/bubble_collapse_validation/2d bubble collapse.xlsx
+++ b/data/bubble_collapse_validation/2d bubble collapse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\oluse\diffuse_vs_GFM_MMS\data\bubble_collapse_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A330E16-10C1-4F05-A963-D010DB009C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5A6E83-F5DA-4C01-9B9F-4EF4670B3651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{EDC50580-E04D-44B0-82D6-6934DBA8A6C2}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EDC50580-E04D-44B0-82D6-6934DBA8A6C2}"/>
   </bookViews>
   <sheets>
     <sheet name="GFM" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -142,11 +142,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -276,6 +275,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:trendlineType val="linear"/>
+            <c:intercept val="-345"/>
             <c:dispRSqr val="1"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
@@ -746,6 +746,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:trendlineType val="linear"/>
+            <c:intercept val="-345"/>
             <c:dispRSqr val="1"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
@@ -787,62 +788,50 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>GFM!$O$4:$O$21</c:f>
+              <c:f>GFM!$O$8:$O$21</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
-                  <c:v>138.56</c:v>
+                  <c:v>181.03</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>161.72999999999999</c:v>
+                  <c:v>184.24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>175.55</c:v>
+                  <c:v>187.98</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>177.88</c:v>
+                  <c:v>192.09</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>181.03</c:v>
+                  <c:v>196.09</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>184.24</c:v>
+                  <c:v>200.71</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>187.98</c:v>
+                  <c:v>204.57</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>192.09</c:v>
+                  <c:v>208.43</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>196.09</c:v>
+                  <c:v>211.9</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>200.71</c:v>
+                  <c:v>214.61</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>204.57</c:v>
+                  <c:v>218.08</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>208.43</c:v>
+                  <c:v>221.61</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>211.9</c:v>
+                  <c:v>225.54</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>214.61</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>218.08</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>221.61</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>225.54</c:v>
-                </c:pt>
-                <c:pt idx="17">
                   <c:v>229.28</c:v>
                 </c:pt>
               </c:numCache>
@@ -6266,9 +6255,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>336386</xdr:colOff>
+      <xdr:colOff>333211</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>103866</xdr:rowOff>
+      <xdr:rowOff>107041</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7009,13 +6998,15 @@
       <c r="R2" t="s">
         <v>6</v>
       </c>
-      <c r="S2" s="3">
-        <v>104</v>
-      </c>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3">
-        <v>176</v>
+      <c r="S2" s="2">
+        <f>M23</f>
+        <v>109.01037519872251</v>
+      </c>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2">
+        <f>O23</f>
+        <v>143.67794726052384</v>
       </c>
     </row>
     <row r="3" spans="6:22" x14ac:dyDescent="0.35">
@@ -7031,7 +7022,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="J3" t="e">
-        <f t="shared" ref="J3:J21" si="2">150-O3</f>
+        <f t="shared" ref="J3" si="2">150-O3</f>
         <v>#VALUE!</v>
       </c>
       <c r="L3">
@@ -7105,7 +7096,7 @@
       </c>
       <c r="S4" s="1">
         <f>((S2-S3)/S2)*100</f>
-        <v>-63.46153846153846</v>
+        <v>-55.948458749999993</v>
       </c>
       <c r="T4" s="1" t="e">
         <f t="shared" ref="T4:V4" si="5">((T2-T3)/T2)*100</f>
@@ -7117,7 +7108,7 @@
       </c>
       <c r="V4" s="1">
         <f t="shared" si="5"/>
-        <v>17.613636363636363</v>
+        <v>-0.9201500749999949</v>
       </c>
     </row>
     <row r="5" spans="6:22" x14ac:dyDescent="0.35">
@@ -7179,16 +7170,16 @@
       <c r="L6">
         <v>35.274999999999999</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6">
         <v>136.58000000000001</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6">
         <v>136.58000000000001</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6">
         <v>175.55</v>
       </c>
-      <c r="P6" s="2" t="s">
+      <c r="P6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -7740,16 +7731,16 @@
       </c>
     </row>
     <row r="23" spans="6:16" x14ac:dyDescent="0.35">
-      <c r="H23" t="s">
+      <c r="L23" t="s">
         <v>14</v>
       </c>
-      <c r="I23">
-        <f>1.8531^-1*$R$8</f>
-        <v>155.44758321872769</v>
-      </c>
-      <c r="J23">
-        <f>2.4716^-1*$R$8</f>
-        <v>116.5479513119535</v>
+      <c r="M23">
+        <f>2.6425^-1*$R$8</f>
+        <v>109.01037519872251</v>
+      </c>
+      <c r="O23">
+        <f>2.0049^-1*$R$8</f>
+        <v>143.67794726052384</v>
       </c>
     </row>
   </sheetData>
@@ -7848,19 +7839,19 @@
       <c r="R2" t="s">
         <v>6</v>
       </c>
-      <c r="S2" s="3">
+      <c r="S2" s="2">
         <f>M23</f>
         <v>129.43604424292261</v>
       </c>
-      <c r="T2" s="3">
+      <c r="T2" s="2">
         <f>N23</f>
         <v>214.12318179039934</v>
       </c>
-      <c r="U2" s="3">
+      <c r="U2" s="2">
         <f>P23</f>
         <v>446.46608255211447</v>
       </c>
-      <c r="V2" s="3">
+      <c r="V2" s="2">
         <f>O23</f>
         <v>135.65336306222002</v>
       </c>
@@ -7878,7 +7869,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="J3" t="e">
-        <f t="shared" ref="J3:J21" si="2">150-O3</f>
+        <f t="shared" ref="J3" si="2">150-O3</f>
         <v>#VALUE!</v>
       </c>
       <c r="L3">
@@ -7932,16 +7923,16 @@
         <f t="shared" ref="J4:J12" si="4">ABS(150-O4)</f>
         <v>26.169999999999987</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>21.164999999999999</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="3">
         <v>125.45</v>
       </c>
       <c r="N4" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="3">
         <v>176.17</v>
       </c>
       <c r="P4" t="s">
@@ -7990,13 +7981,13 @@
       <c r="L5">
         <v>28.22</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="3">
         <v>129.4</v>
       </c>
       <c r="N5" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="4">
+      <c r="O5" s="3">
         <v>176.59</v>
       </c>
       <c r="P5" t="s">
@@ -8026,16 +8017,16 @@
       <c r="L6">
         <v>35.274999999999999</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6">
         <v>133.63999999999999</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="N6" t="s">
         <v>18</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6">
         <v>176.86</v>
       </c>
-      <c r="P6" s="2" t="s">
+      <c r="P6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -8062,16 +8053,16 @@
       <c r="L7">
         <v>42.33</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7">
         <v>138.29</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N7" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7">
         <v>179.19</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="P7" t="s">
         <v>18</v>
       </c>
       <c r="R7" t="s">
@@ -8101,13 +8092,13 @@
       <c r="L8">
         <v>49.384999999999998</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8">
         <v>142.88</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="N8" t="s">
         <v>18</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8">
         <v>181.85</v>
       </c>
       <c r="P8">
@@ -8141,16 +8132,16 @@
       <c r="L9">
         <v>56.44</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9">
         <v>147.04</v>
       </c>
       <c r="N9">
         <v>147.32</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9">
         <v>184.66</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9">
         <v>187.67</v>
       </c>
     </row>
@@ -8177,13 +8168,13 @@
       <c r="L10">
         <v>63.494999999999997</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10">
         <v>151.01</v>
       </c>
       <c r="N10">
         <v>153.19999999999999</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10">
         <v>187.8</v>
       </c>
       <c r="P10">
@@ -8213,13 +8204,13 @@
       <c r="L11">
         <v>70.55</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11">
         <v>154.25</v>
       </c>
       <c r="N11">
         <v>157.22999999999999</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11">
         <v>191.57</v>
       </c>
       <c r="P11">
@@ -8249,13 +8240,13 @@
       <c r="L12">
         <v>77.605000000000004</v>
       </c>
-      <c r="M12" s="2">
+      <c r="M12">
         <v>156.84</v>
       </c>
       <c r="N12">
         <v>162.97999999999999</v>
       </c>
-      <c r="O12" s="2">
+      <c r="O12">
         <v>195.27</v>
       </c>
       <c r="P12">
@@ -8285,13 +8276,13 @@
       <c r="L13">
         <v>84.66</v>
       </c>
-      <c r="M13" s="2">
+      <c r="M13">
         <v>159.30000000000001</v>
       </c>
       <c r="N13">
         <v>167.88</v>
       </c>
-      <c r="O13" s="2">
+      <c r="O13">
         <v>198.82</v>
       </c>
       <c r="P13">
@@ -8321,13 +8312,13 @@
       <c r="L14">
         <v>91.715000000000003</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14">
         <v>161.99</v>
       </c>
       <c r="N14">
         <v>173.95</v>
       </c>
-      <c r="O14" s="2">
+      <c r="O14">
         <v>202.84</v>
       </c>
       <c r="P14">
@@ -8357,13 +8348,13 @@
       <c r="L15">
         <v>98.77</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15">
         <v>164.48</v>
       </c>
       <c r="N15">
         <v>179.2</v>
       </c>
-      <c r="O15" s="2">
+      <c r="O15">
         <v>205.77</v>
       </c>
       <c r="P15">

</xml_diff>